<commit_message>
feat: Update penalty values in constraints and adjust shift timings for improved scheduling logic
</commit_message>
<xml_diff>
--- a/out/Template.xlsx
+++ b/out/Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/guiarcoelho/Desktop/Pharmacy_Scheduler_Portugal/out/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC091E45-ADFF-9846-96F2-24A08A713723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA9B091-BA23-3744-B899-CC298DA106EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="4" r:id="rId1"/>
@@ -465,6 +465,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -472,9 +475,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1031,7 +1031,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:90" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
@@ -1303,7 +1303,7 @@
       </c>
     </row>
     <row r="2" spans="1:90" x14ac:dyDescent="0.2">
-      <c r="A2" s="18"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="14">
         <v>46054</v>
       </c>
@@ -3298,7 +3298,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="20" t="s">
         <v>69</v>
       </c>
       <c r="B2" s="11" t="s">
@@ -3315,7 +3315,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="19"/>
+      <c r="A3" s="20"/>
       <c r="B3" s="11" t="s">
         <v>13</v>
       </c>
@@ -3330,7 +3330,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="19"/>
+      <c r="A4" s="20"/>
       <c r="B4" s="11" t="s">
         <v>3</v>
       </c>
@@ -3345,7 +3345,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="21" t="s">
         <v>70</v>
       </c>
       <c r="B5" s="6" t="s">
@@ -3362,7 +3362,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="20"/>
+      <c r="A6" s="21"/>
       <c r="B6" s="6" t="s">
         <v>12</v>
       </c>
@@ -3377,7 +3377,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="20"/>
+      <c r="A7" s="21"/>
       <c r="B7" s="6" t="s">
         <v>4</v>
       </c>
@@ -3392,7 +3392,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="20" t="s">
         <v>71</v>
       </c>
       <c r="B8" s="11" t="s">
@@ -3409,7 +3409,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="19"/>
+      <c r="A9" s="20"/>
       <c r="B9" s="11" t="s">
         <v>6</v>
       </c>
@@ -3424,7 +3424,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="19"/>
+      <c r="A10" s="20"/>
       <c r="B10" s="11" t="s">
         <v>11</v>
       </c>
@@ -3439,7 +3439,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="19"/>
+      <c r="A11" s="20"/>
       <c r="B11" s="11" t="s">
         <v>7</v>
       </c>
@@ -3454,7 +3454,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="19"/>
+      <c r="A12" s="20"/>
       <c r="B12" s="11" t="s">
         <v>15</v>
       </c>
@@ -3465,11 +3465,11 @@
         <v>0</v>
       </c>
       <c r="E12" s="12">
-        <v>0.35416666666666669</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="20" t="s">
+      <c r="A13" s="21" t="s">
         <v>72</v>
       </c>
       <c r="B13" s="6" t="s">
@@ -3486,7 +3486,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="20"/>
+      <c r="A14" s="21"/>
       <c r="B14" s="6" t="s">
         <v>10</v>
       </c>
@@ -3501,7 +3501,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="20"/>
+      <c r="A15" s="21"/>
       <c r="B15" s="6" t="s">
         <v>9</v>
       </c>
@@ -3516,7 +3516,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="20"/>
+      <c r="A16" s="21"/>
       <c r="B16" s="6" t="s">
         <v>17</v>
       </c>
@@ -3531,7 +3531,7 @@
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" s="20"/>
+      <c r="A17" s="21"/>
       <c r="B17" s="6" t="s">
         <v>16</v>
       </c>
@@ -3601,85 +3601,85 @@
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="F1" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="G1" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="H1" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="I1" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="J1" s="21" t="s">
+      <c r="J1" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="K1" s="21" t="s">
+      <c r="K1" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="L1" s="21" t="s">
+      <c r="L1" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="M1" s="21" t="s">
+      <c r="M1" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="21" t="s">
+      <c r="N1" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="21" t="s">
+      <c r="O1" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="21" t="s">
+      <c r="P1" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="21" t="s">
+      <c r="Q1" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="21" t="s">
+      <c r="R1" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="S1" s="21" t="s">
+      <c r="S1" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="T1" s="21" t="s">
+      <c r="T1" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="U1" s="21" t="s">
+      <c r="U1" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="V1" s="21" t="s">
+      <c r="V1" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="W1" s="21" t="s">
+      <c r="W1" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="X1" s="21" t="s">
+      <c r="X1" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="Y1" s="21" t="s">
+      <c r="Y1" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="Z1" s="21" t="s">
+      <c r="Z1" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="AA1" s="21" t="s">
+      <c r="AA1" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="AB1" s="21" t="s">
+      <c r="AB1" s="18" t="s">
         <v>43</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Update Template.xlsx for improved scheduling layout and data presentation
</commit_message>
<xml_diff>
--- a/out/Template.xlsx
+++ b/out/Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/guiarcoelho/Desktop/Pharmacy_Scheduler_Portugal/out/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA9B091-BA23-3744-B899-CC298DA106EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5531408E-8435-CB4C-AFD8-000643F981B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="4" r:id="rId1"/>

</xml_diff>